<commit_message>
Renamed 'global' to 'unallocated' in figure 3, because the term was misleading. We do not know where the emissions are from, because they are added from the bottom-up calculations.
</commit_message>
<xml_diff>
--- a/output/FullResults_Tables.xlsx
+++ b/output/FullResults_Tables.xlsx
@@ -102,13 +102,13 @@
     <t>Europe</t>
   </si>
   <si>
-    <t>Global</t>
-  </si>
-  <si>
     <t>Middle East</t>
   </si>
   <si>
     <t>Netherlands</t>
+  </si>
+  <si>
+    <t>Unallocated</t>
   </si>
 </sst>
 </file>
@@ -1394,19 +1394,19 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>219.73</v>
+        <v>259.4625128535352</v>
       </c>
       <c r="C7">
-        <v>24.6529</v>
+        <v>143.5487102776829</v>
       </c>
       <c r="D7">
-        <v>0.1713</v>
+        <v>11.16237613197063</v>
       </c>
       <c r="E7">
-        <v>1.6049</v>
+        <v>113.44803780191</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>24.74474248431348</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1414,19 +1414,19 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>259.4625128535352</v>
+        <v>70.86450767155036</v>
       </c>
       <c r="C8">
-        <v>143.5487102776829</v>
+        <v>10.50689156446671</v>
       </c>
       <c r="D8">
-        <v>11.16237613197063</v>
+        <v>0.2020725477166485</v>
       </c>
       <c r="E8">
-        <v>113.44803780191</v>
+        <v>5.59775099657913</v>
       </c>
       <c r="F8">
-        <v>24.74474248431348</v>
+        <v>6.521566738846172</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1434,19 +1434,19 @@
         <v>29</v>
       </c>
       <c r="B9">
-        <v>70.86450767155036</v>
+        <v>219.73</v>
       </c>
       <c r="C9">
-        <v>10.50689156446671</v>
+        <v>24.6529</v>
       </c>
       <c r="D9">
-        <v>0.2020725477166485</v>
+        <v>0.1713</v>
       </c>
       <c r="E9">
-        <v>5.59775099657913</v>
+        <v>1.6049</v>
       </c>
       <c r="F9">
-        <v>6.521566738846172</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1484,7 +1484,7 @@
         <v>22</v>
       </c>
       <c r="B2">
-        <v>1.998352710653227</v>
+        <v>1.998352710653228</v>
       </c>
       <c r="C2">
         <v>1.538449817132225</v>
@@ -1504,7 +1504,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>3.404173560934444</v>
+        <v>3.404173560934445</v>
       </c>
       <c r="C3">
         <v>3.658446568725746</v>
@@ -1544,7 +1544,7 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>45.14860140579809</v>
+        <v>45.1486014057981</v>
       </c>
       <c r="C5">
         <v>59.2369489711885</v>
@@ -1564,7 +1564,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>19.86981441161389</v>
+        <v>19.8698144116139</v>
       </c>
       <c r="C6">
         <v>16.65971505231471</v>
@@ -1584,19 +1584,19 @@
         <v>27</v>
       </c>
       <c r="B7">
-        <v>4.563742804988675</v>
+        <v>5.388978183223061</v>
       </c>
       <c r="C7">
-        <v>0.9479847841873641</v>
+        <v>5.519918270587384</v>
       </c>
       <c r="D7">
-        <v>0.3680494064746837</v>
+        <v>23.98310513846447</v>
       </c>
       <c r="E7">
-        <v>0.05829316005112441</v>
+        <v>4.120658374398872</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>2.945178204383617</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1604,19 +1604,19 @@
         <v>28</v>
       </c>
       <c r="B8">
-        <v>5.38897818322306</v>
+        <v>1.471839926341887</v>
       </c>
       <c r="C8">
-        <v>5.519918270587384</v>
+        <v>0.4040244081718989</v>
       </c>
       <c r="D8">
-        <v>23.98310513846447</v>
+        <v>0.4341662653353163</v>
       </c>
       <c r="E8">
-        <v>4.120658374398872</v>
+        <v>0.2033214497912196</v>
       </c>
       <c r="F8">
-        <v>2.945178204383617</v>
+        <v>0.7762124107720646</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1624,19 +1624,19 @@
         <v>29</v>
       </c>
       <c r="B9">
-        <v>1.471839926341887</v>
+        <v>4.563742804988676</v>
       </c>
       <c r="C9">
-        <v>0.4040244081718989</v>
+        <v>0.9479847841873641</v>
       </c>
       <c r="D9">
-        <v>0.4341662653353163</v>
+        <v>0.3680494064746837</v>
       </c>
       <c r="E9">
-        <v>0.2033214497912196</v>
+        <v>0.05829316005112441</v>
       </c>
       <c r="F9">
-        <v>0.7762124107720646</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aligned legends and bars in the graphs in alphabetical order. Synchronised Figure 1 and 2 with Figure 3, buy changing terminology from 'other' to 'Unallocated'. Put Denmark first in graph 3. Increased Dpi of graphs to 600
</commit_message>
<xml_diff>
--- a/output/FullResults_Tables.xlsx
+++ b/output/FullResults_Tables.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="29">
   <si>
     <t>Global warming (ktCO2eq)</t>
   </si>
@@ -54,9 +54,6 @@
     <t>Operational impacts</t>
   </si>
   <si>
-    <t>Other</t>
-  </si>
-  <si>
     <t>Pharmaceuticals and chemical products</t>
   </si>
   <si>
@@ -66,6 +63,9 @@
     <t>Transport</t>
   </si>
   <si>
+    <t>Unallocated</t>
+  </si>
+  <si>
     <t>Hotspot</t>
   </si>
   <si>
@@ -87,28 +87,25 @@
     <t>Region</t>
   </si>
   <si>
+    <t>Netherlands</t>
+  </si>
+  <si>
+    <t>Middle East</t>
+  </si>
+  <si>
+    <t>Europe</t>
+  </si>
+  <si>
+    <t>Asia and Pacific</t>
+  </si>
+  <si>
+    <t>America</t>
+  </si>
+  <si>
     <t>Africa</t>
   </si>
   <si>
-    <t>America</t>
-  </si>
-  <si>
-    <t>Asia and Pacific</t>
-  </si>
-  <si>
     <t>Denmark</t>
-  </si>
-  <si>
-    <t>Europe</t>
-  </si>
-  <si>
-    <t>Middle East</t>
-  </si>
-  <si>
-    <t>Netherlands</t>
-  </si>
-  <si>
-    <t>Unallocated</t>
   </si>
 </sst>
 </file>
@@ -594,19 +591,19 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>345.0932546254422</v>
+        <v>850.1357460021289</v>
       </c>
       <c r="C7">
-        <v>730.293714813014</v>
+        <v>1214.789496785072</v>
       </c>
       <c r="D7">
-        <v>1.854354511665176</v>
+        <v>18.05538349698451</v>
       </c>
       <c r="E7">
-        <v>150.4964365867146</v>
+        <v>805.9736325057729</v>
       </c>
       <c r="F7">
-        <v>71.89171149077825</v>
+        <v>235.6814660850752</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -614,19 +611,19 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>850.1357460021289</v>
+        <v>650.5283522565269</v>
       </c>
       <c r="C8">
-        <v>1214.789496785072</v>
+        <v>228.5771111911285</v>
       </c>
       <c r="D8">
-        <v>18.05538349698451</v>
+        <v>7.363211691016988</v>
       </c>
       <c r="E8">
-        <v>805.9736325057729</v>
+        <v>424.6312600729522</v>
       </c>
       <c r="F8">
-        <v>235.6814660850752</v>
+        <v>85.32465855958648</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -634,19 +631,19 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>650.5283522565269</v>
+        <v>1855.119022051182</v>
       </c>
       <c r="C9">
-        <v>228.5771111911285</v>
+        <v>138.5532218937953</v>
       </c>
       <c r="D9">
-        <v>7.363211691016988</v>
+        <v>3.722327246233987</v>
       </c>
       <c r="E9">
-        <v>424.6312600729522</v>
+        <v>257.7487519531698</v>
       </c>
       <c r="F9">
-        <v>85.32465855958648</v>
+        <v>60.91403759533326</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -654,19 +651,19 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>1855.119022051182</v>
+        <v>345.0932546254422</v>
       </c>
       <c r="C10">
-        <v>138.5532218937953</v>
+        <v>730.293714813014</v>
       </c>
       <c r="D10">
-        <v>3.722327246233987</v>
+        <v>1.854354511665176</v>
       </c>
       <c r="E10">
-        <v>257.7487519531698</v>
+        <v>150.4964365867146</v>
       </c>
       <c r="F10">
-        <v>60.91403759533326</v>
+        <v>71.89171149077825</v>
       </c>
     </row>
   </sheetData>
@@ -704,7 +701,7 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>5.966408293881514</v>
+        <v>5.966408293881512</v>
       </c>
       <c r="C2">
         <v>3.081643178684756</v>
@@ -747,7 +744,7 @@
         <v>11.21651011143046</v>
       </c>
       <c r="C4">
-        <v>0.9479847841873625</v>
+        <v>0.9479847841873624</v>
       </c>
       <c r="D4">
         <v>0.3680494064746833</v>
@@ -764,10 +761,10 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>4.652491596644828</v>
+        <v>4.652491596644827</v>
       </c>
       <c r="C5">
-        <v>6.518765060407505</v>
+        <v>6.518765060407504</v>
       </c>
       <c r="D5">
         <v>5.636234596423445</v>
@@ -804,19 +801,19 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>7.167509776854899</v>
+        <v>17.65712945545026</v>
       </c>
       <c r="C7">
-        <v>28.08218625923938</v>
+        <v>46.71263660432935</v>
       </c>
       <c r="D7">
-        <v>3.984203604273317</v>
+        <v>38.79318843980117</v>
       </c>
       <c r="E7">
-        <v>5.466329905335694</v>
+        <v>29.27456536646843</v>
       </c>
       <c r="F7">
-        <v>8.556722782332464</v>
+        <v>28.05136960026833</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -824,19 +821,19 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>17.65712945545026</v>
+        <v>13.51132849577352</v>
       </c>
       <c r="C8">
-        <v>46.71263660432935</v>
+        <v>8.789538894924846</v>
       </c>
       <c r="D8">
-        <v>38.79318843980117</v>
+        <v>15.82034846833772</v>
       </c>
       <c r="E8">
-        <v>29.27456536646843</v>
+        <v>15.42345193229687</v>
       </c>
       <c r="F8">
-        <v>28.05136960026833</v>
+        <v>10.15554414621502</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -844,19 +841,19 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>13.51132849577352</v>
+        <v>38.53040750452572</v>
       </c>
       <c r="C9">
-        <v>8.789538894924847</v>
+        <v>5.327825373706673</v>
       </c>
       <c r="D9">
-        <v>15.82034846833772</v>
+        <v>7.997666863286404</v>
       </c>
       <c r="E9">
-        <v>15.42345193229687</v>
+        <v>9.361947317953581</v>
       </c>
       <c r="F9">
-        <v>10.15554414621502</v>
+        <v>7.250133881187448</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -864,19 +861,19 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>38.53040750452573</v>
+        <v>7.167509776854898</v>
       </c>
       <c r="C10">
-        <v>5.327825373706674</v>
+        <v>28.08218625923937</v>
       </c>
       <c r="D10">
-        <v>7.997666863286404</v>
+        <v>3.984203604273317</v>
       </c>
       <c r="E10">
-        <v>9.361947317953581</v>
+        <v>5.466329905335694</v>
       </c>
       <c r="F10">
-        <v>7.250133881187448</v>
+        <v>8.556722782332464</v>
       </c>
     </row>
   </sheetData>
@@ -1011,42 +1008,42 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B7">
-        <v>1311.799524406422</v>
+        <v>260.7946795106796</v>
       </c>
       <c r="C7">
-        <v>159.1172301778207</v>
+        <v>32.11769369483017</v>
       </c>
       <c r="D7">
-        <v>2.185348717813712</v>
+        <v>1.671353709306039</v>
       </c>
       <c r="E7">
-        <v>29.96306735323413</v>
+        <v>0.366652289793865</v>
       </c>
       <c r="F7">
-        <v>79.2664639042676</v>
+        <v>111.5663742786052</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B8">
-        <v>260.7946795106796</v>
+        <v>2193.540840045223</v>
       </c>
       <c r="C8">
-        <v>32.11769369483017</v>
+        <v>15.55572396927131</v>
       </c>
       <c r="D8">
-        <v>1.671353709306039</v>
+        <v>0.04142330350065114</v>
       </c>
       <c r="E8">
-        <v>0.366652289793865</v>
+        <v>3.023278572901645</v>
       </c>
       <c r="F8">
-        <v>111.5663742786052</v>
+        <v>5.476472762726005</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1054,19 +1051,19 @@
         <v>14</v>
       </c>
       <c r="B9">
-        <v>2193.540840045223</v>
+        <v>1311.799524406422</v>
       </c>
       <c r="C9">
-        <v>15.55572396927131</v>
+        <v>159.1172301778207</v>
       </c>
       <c r="D9">
-        <v>0.04142330350065114</v>
+        <v>2.185348717813712</v>
       </c>
       <c r="E9">
-        <v>3.023278572901645</v>
+        <v>29.96306735323413</v>
       </c>
       <c r="F9">
-        <v>5.476472762726005</v>
+        <v>79.2664639042676</v>
       </c>
     </row>
   </sheetData>
@@ -1104,7 +1101,7 @@
         <v>16</v>
       </c>
       <c r="B2">
-        <v>7.27408057431946</v>
+        <v>7.274080574319458</v>
       </c>
       <c r="C2">
         <v>1.043794641200905</v>
@@ -1124,7 +1121,7 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>5.508830043839599</v>
+        <v>5.508830043839598</v>
       </c>
       <c r="C3">
         <v>0.1930722495924435</v>
@@ -1144,7 +1141,7 @@
         <v>18</v>
       </c>
       <c r="B4">
-        <v>7.533734581037105</v>
+        <v>7.533734581037104</v>
       </c>
       <c r="C4">
         <v>0.2985713274993635</v>
@@ -1176,7 +1173,7 @@
         <v>0.01142566112127595</v>
       </c>
       <c r="F5">
-        <v>25.61184831342349</v>
+        <v>25.61184831342348</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1196,47 +1193,47 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>20.93131406985195</v>
+        <v>20.93131406985194</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B7">
-        <v>27.24578182814078</v>
+        <v>5.416646985828931</v>
       </c>
       <c r="C7">
-        <v>6.118578873504235</v>
+        <v>1.235030561349352</v>
       </c>
       <c r="D7">
-        <v>4.695366599717145</v>
+        <v>3.591014248215692</v>
       </c>
       <c r="E7">
-        <v>1.088318201037259</v>
+        <v>0.01331754041501963</v>
       </c>
       <c r="F7">
-        <v>9.434483384799982</v>
+        <v>13.27889567150487</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B8">
-        <v>5.416646985828932</v>
+        <v>45.55935114096937</v>
       </c>
       <c r="C8">
-        <v>1.235030561349352</v>
+        <v>0.5981685574471104</v>
       </c>
       <c r="D8">
-        <v>3.591014248215692</v>
+        <v>0.08900071376319511</v>
       </c>
       <c r="E8">
-        <v>0.01331754041501963</v>
+        <v>0.1098114908899561</v>
       </c>
       <c r="F8">
-        <v>13.27889567150488</v>
+        <v>0.6518228358167801</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1244,19 +1241,19 @@
         <v>14</v>
       </c>
       <c r="B9">
-        <v>45.55935114096938</v>
+        <v>27.24578182814077</v>
       </c>
       <c r="C9">
-        <v>0.5981685574471104</v>
+        <v>6.118578873504235</v>
       </c>
       <c r="D9">
-        <v>0.08900071376319511</v>
+        <v>4.695366599717145</v>
       </c>
       <c r="E9">
-        <v>0.1098114908899561</v>
+        <v>1.088318201037259</v>
       </c>
       <c r="F9">
-        <v>0.6518228358167802</v>
+        <v>9.434483384799982</v>
       </c>
     </row>
   </sheetData>
@@ -1291,162 +1288,162 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B2">
-        <v>96.21445814866054</v>
+        <v>219.73</v>
       </c>
       <c r="C2">
-        <v>40.00828929895873</v>
+        <v>24.6529</v>
       </c>
       <c r="D2">
-        <v>1.977809522791886</v>
+        <v>0.1713</v>
       </c>
       <c r="E2">
-        <v>443.2798730423514</v>
+        <v>1.6049</v>
       </c>
       <c r="F2">
-        <v>36.87581169525912</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3">
-        <v>163.9003529573314</v>
+        <v>70.86450767155036</v>
       </c>
       <c r="C3">
-        <v>95.14004751822378</v>
+        <v>10.50689156446671</v>
       </c>
       <c r="D3">
-        <v>2.97902532656294</v>
+        <v>0.2020725477166485</v>
       </c>
       <c r="E3">
-        <v>379.3092360518981</v>
+        <v>5.59775099657913</v>
       </c>
       <c r="F3">
-        <v>93.97507235259351</v>
+        <v>6.521566738846172</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4">
-        <v>874.0824791153266</v>
+        <v>259.4625128535352</v>
       </c>
       <c r="C4">
-        <v>312.9645422390495</v>
+        <v>143.5487102776829</v>
       </c>
       <c r="D4">
-        <v>21.79579330166932</v>
+        <v>11.16237613197063</v>
       </c>
       <c r="E4">
-        <v>808.3941676249243</v>
+        <v>113.44803780191</v>
       </c>
       <c r="F4">
-        <v>154.5922928425451</v>
+        <v>24.74474248431348</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5">
-        <v>2173.764519782274</v>
+        <v>956.6696694413642</v>
       </c>
       <c r="C5">
-        <v>1540.491581353462</v>
+        <v>433.2456554830469</v>
       </c>
       <c r="D5">
-        <v>3.881355370673937</v>
+        <v>4.37293217641548</v>
       </c>
       <c r="E5">
-        <v>242.3632615404337</v>
+        <v>759.1559706626429</v>
       </c>
       <c r="F5">
-        <v>387.3329918255739</v>
+        <v>136.135629025102</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6">
-        <v>956.6696694413642</v>
+        <v>874.0824791153266</v>
       </c>
       <c r="C6">
-        <v>433.2456554830469</v>
+        <v>312.9645422390495</v>
       </c>
       <c r="D6">
-        <v>4.37293217641548</v>
+        <v>21.79579330166932</v>
       </c>
       <c r="E6">
-        <v>759.1559706626429</v>
+        <v>808.3941676249243</v>
       </c>
       <c r="F6">
-        <v>136.135629025102</v>
+        <v>154.5922928425451</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B7">
-        <v>259.4625128535352</v>
+        <v>163.9003529573314</v>
       </c>
       <c r="C7">
-        <v>143.5487102776829</v>
+        <v>95.14004751822378</v>
       </c>
       <c r="D7">
-        <v>11.16237613197063</v>
+        <v>2.97902532656294</v>
       </c>
       <c r="E7">
-        <v>113.44803780191</v>
+        <v>379.3092360518981</v>
       </c>
       <c r="F7">
-        <v>24.74474248431348</v>
+        <v>93.97507235259351</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8">
-        <v>70.86450767155036</v>
+        <v>96.21445814866054</v>
       </c>
       <c r="C8">
-        <v>10.50689156446671</v>
+        <v>40.00828929895873</v>
       </c>
       <c r="D8">
-        <v>0.2020725477166485</v>
+        <v>1.977809522791886</v>
       </c>
       <c r="E8">
-        <v>5.59775099657913</v>
+        <v>443.2798730423514</v>
       </c>
       <c r="F8">
-        <v>6.521566738846172</v>
+        <v>36.87581169525912</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9">
-        <v>219.73</v>
+        <v>2173.764519782274</v>
       </c>
       <c r="C9">
-        <v>24.6529</v>
+        <v>1540.491581353462</v>
       </c>
       <c r="D9">
-        <v>0.1713</v>
+        <v>3.881355370673937</v>
       </c>
       <c r="E9">
-        <v>1.6049</v>
+        <v>242.3632615404337</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>387.3329918255739</v>
       </c>
     </row>
   </sheetData>
@@ -1481,162 +1478,162 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B2">
-        <v>1.998352710653228</v>
+        <v>4.563742804988676</v>
       </c>
       <c r="C2">
-        <v>1.538449817132225</v>
+        <v>0.9479847841873641</v>
       </c>
       <c r="D2">
-        <v>4.24945488023077</v>
+        <v>0.3680494064746836</v>
       </c>
       <c r="E2">
-        <v>16.10080664633304</v>
+        <v>0.0582931600511244</v>
       </c>
       <c r="F2">
-        <v>4.389046963922964</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3">
-        <v>3.404173560934445</v>
+        <v>1.471839926341887</v>
       </c>
       <c r="C3">
-        <v>3.658446568725746</v>
+        <v>0.4040244081718989</v>
       </c>
       <c r="D3">
-        <v>6.400633411059784</v>
+        <v>0.4341662653353162</v>
       </c>
       <c r="E3">
-        <v>13.77726587702849</v>
+        <v>0.2033214497912196</v>
       </c>
       <c r="F3">
-        <v>11.18513700531286</v>
+        <v>0.7762124107720648</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4">
-        <v>18.15449699644671</v>
+        <v>5.388978183223061</v>
       </c>
       <c r="C4">
-        <v>12.03451212769218</v>
+        <v>5.519918270587384</v>
       </c>
       <c r="D4">
-        <v>46.82970687871734</v>
+        <v>23.98310513846447</v>
       </c>
       <c r="E4">
-        <v>29.36248401629709</v>
+        <v>4.120658374398871</v>
       </c>
       <c r="F4">
-        <v>18.39994300745641</v>
+        <v>2.945178204383618</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5">
-        <v>45.1486014057981</v>
+        <v>19.8698144116139</v>
       </c>
       <c r="C5">
-        <v>59.2369489711885</v>
+        <v>16.65971505231471</v>
       </c>
       <c r="D5">
-        <v>8.339349331546224</v>
+        <v>9.395534688171416</v>
       </c>
       <c r="E5">
-        <v>8.80311570533306</v>
+        <v>27.57405477076711</v>
       </c>
       <c r="F5">
-        <v>46.10129550091487</v>
+        <v>16.2031869072372</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6">
-        <v>19.8698144116139</v>
+        <v>18.15449699644671</v>
       </c>
       <c r="C6">
-        <v>16.65971505231471</v>
+        <v>12.03451212769218</v>
       </c>
       <c r="D6">
-        <v>9.395534688171418</v>
+        <v>46.82970687871733</v>
       </c>
       <c r="E6">
-        <v>27.57405477076711</v>
+        <v>29.36248401629709</v>
       </c>
       <c r="F6">
-        <v>16.2031869072372</v>
+        <v>18.39994300745641</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B7">
-        <v>5.388978183223061</v>
+        <v>3.404173560934445</v>
       </c>
       <c r="C7">
-        <v>5.519918270587384</v>
+        <v>3.658446568725746</v>
       </c>
       <c r="D7">
-        <v>23.98310513846447</v>
+        <v>6.400633411059783</v>
       </c>
       <c r="E7">
-        <v>4.120658374398872</v>
+        <v>13.77726587702849</v>
       </c>
       <c r="F7">
-        <v>2.945178204383617</v>
+        <v>11.18513700531286</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8">
-        <v>1.471839926341887</v>
+        <v>1.998352710653228</v>
       </c>
       <c r="C8">
-        <v>0.4040244081718989</v>
+        <v>1.538449817132225</v>
       </c>
       <c r="D8">
-        <v>0.4341662653353163</v>
+        <v>4.249454880230769</v>
       </c>
       <c r="E8">
-        <v>0.2033214497912196</v>
+        <v>16.10080664633304</v>
       </c>
       <c r="F8">
-        <v>0.7762124107720646</v>
+        <v>4.389046963922966</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9">
-        <v>4.563742804988676</v>
+        <v>45.1486014057981</v>
       </c>
       <c r="C9">
-        <v>0.9479847841873641</v>
+        <v>59.2369489711885</v>
       </c>
       <c r="D9">
-        <v>0.3680494064746837</v>
+        <v>8.339349331546222</v>
       </c>
       <c r="E9">
-        <v>0.05829316005112441</v>
+        <v>8.803115705333058</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>46.10129550091488</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merged Netherlands into Europe category in figure3 results
</commit_message>
<xml_diff>
--- a/output/FullResults_Tables.xlsx
+++ b/output/FullResults_Tables.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="28">
   <si>
     <t>Global warming (ktCO2eq)</t>
   </si>
@@ -85,9 +85,6 @@
   </si>
   <si>
     <t>Region</t>
-  </si>
-  <si>
-    <t>Netherlands</t>
   </si>
   <si>
     <t>Middle East</t>
@@ -1263,7 +1260,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1311,19 +1308,19 @@
         <v>22</v>
       </c>
       <c r="B3">
-        <v>70.86450767155036</v>
+        <v>259.4625128535352</v>
       </c>
       <c r="C3">
-        <v>10.50689156446671</v>
+        <v>143.5487102776829</v>
       </c>
       <c r="D3">
-        <v>0.2020725477166485</v>
+        <v>11.16237613197063</v>
       </c>
       <c r="E3">
-        <v>5.59775099657913</v>
+        <v>113.44803780191</v>
       </c>
       <c r="F3">
-        <v>6.521566738846172</v>
+        <v>24.74474248431348</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1331,19 +1328,19 @@
         <v>23</v>
       </c>
       <c r="B4">
-        <v>259.4625128535352</v>
+        <v>1027.534177112915</v>
       </c>
       <c r="C4">
-        <v>143.5487102776829</v>
+        <v>443.7525470475137</v>
       </c>
       <c r="D4">
-        <v>11.16237613197063</v>
+        <v>4.575004724132128</v>
       </c>
       <c r="E4">
-        <v>113.44803780191</v>
+        <v>764.7537216592217</v>
       </c>
       <c r="F4">
-        <v>24.74474248431348</v>
+        <v>142.6571957639482</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1351,19 +1348,19 @@
         <v>24</v>
       </c>
       <c r="B5">
-        <v>956.6696694413642</v>
+        <v>874.0824791153266</v>
       </c>
       <c r="C5">
-        <v>433.2456554830469</v>
+        <v>312.9645422390495</v>
       </c>
       <c r="D5">
-        <v>4.37293217641548</v>
+        <v>21.79579330166932</v>
       </c>
       <c r="E5">
-        <v>759.1559706626429</v>
+        <v>808.3941676249243</v>
       </c>
       <c r="F5">
-        <v>136.135629025102</v>
+        <v>154.5922928425451</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1371,19 +1368,19 @@
         <v>25</v>
       </c>
       <c r="B6">
-        <v>874.0824791153266</v>
+        <v>163.9003529573314</v>
       </c>
       <c r="C6">
-        <v>312.9645422390495</v>
+        <v>95.14004751822378</v>
       </c>
       <c r="D6">
-        <v>21.79579330166932</v>
+        <v>2.97902532656294</v>
       </c>
       <c r="E6">
-        <v>808.3941676249243</v>
+        <v>379.3092360518981</v>
       </c>
       <c r="F6">
-        <v>154.5922928425451</v>
+        <v>93.97507235259351</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1391,19 +1388,19 @@
         <v>26</v>
       </c>
       <c r="B7">
-        <v>163.9003529573314</v>
+        <v>96.21445814866054</v>
       </c>
       <c r="C7">
-        <v>95.14004751822378</v>
+        <v>40.00828929895873</v>
       </c>
       <c r="D7">
-        <v>2.97902532656294</v>
+        <v>1.977809522791886</v>
       </c>
       <c r="E7">
-        <v>379.3092360518981</v>
+        <v>443.2798730423514</v>
       </c>
       <c r="F7">
-        <v>93.97507235259351</v>
+        <v>36.87581169525912</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1411,38 +1408,18 @@
         <v>27</v>
       </c>
       <c r="B8">
-        <v>96.21445814866054</v>
+        <v>2173.764519782274</v>
       </c>
       <c r="C8">
-        <v>40.00828929895873</v>
+        <v>1540.491581353462</v>
       </c>
       <c r="D8">
-        <v>1.977809522791886</v>
+        <v>3.881355370673937</v>
       </c>
       <c r="E8">
-        <v>443.2798730423514</v>
+        <v>242.3632615404337</v>
       </c>
       <c r="F8">
-        <v>36.87581169525912</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9">
-        <v>2173.764519782274</v>
-      </c>
-      <c r="C9">
-        <v>1540.491581353462</v>
-      </c>
-      <c r="D9">
-        <v>3.881355370673937</v>
-      </c>
-      <c r="E9">
-        <v>242.3632615404337</v>
-      </c>
-      <c r="F9">
         <v>387.3329918255739</v>
       </c>
     </row>
@@ -1453,7 +1430,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1490,7 +1467,7 @@
         <v>0.3680494064746836</v>
       </c>
       <c r="E2">
-        <v>0.0582931600511244</v>
+        <v>0.05829316005112441</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1501,19 +1478,19 @@
         <v>22</v>
       </c>
       <c r="B3">
-        <v>1.471839926341887</v>
+        <v>5.388978183223061</v>
       </c>
       <c r="C3">
-        <v>0.4040244081718989</v>
+        <v>5.519918270587384</v>
       </c>
       <c r="D3">
-        <v>0.4341662653353162</v>
+        <v>23.98310513846447</v>
       </c>
       <c r="E3">
-        <v>0.2033214497912196</v>
+        <v>4.120658374398872</v>
       </c>
       <c r="F3">
-        <v>0.7762124107720648</v>
+        <v>2.945178204383618</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1521,19 +1498,19 @@
         <v>23</v>
       </c>
       <c r="B4">
-        <v>5.388978183223061</v>
+        <v>21.34165433795578</v>
       </c>
       <c r="C4">
-        <v>5.519918270587384</v>
+        <v>17.06373946048661</v>
       </c>
       <c r="D4">
-        <v>23.98310513846447</v>
+        <v>9.829700953506732</v>
       </c>
       <c r="E4">
-        <v>4.120658374398871</v>
+        <v>27.77737622055832</v>
       </c>
       <c r="F4">
-        <v>2.945178204383618</v>
+        <v>16.97939931800926</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1541,19 +1518,19 @@
         <v>24</v>
       </c>
       <c r="B5">
-        <v>19.8698144116139</v>
+        <v>18.15449699644671</v>
       </c>
       <c r="C5">
-        <v>16.65971505231471</v>
+        <v>12.03451212769218</v>
       </c>
       <c r="D5">
-        <v>9.395534688171416</v>
+        <v>46.82970687871733</v>
       </c>
       <c r="E5">
-        <v>27.57405477076711</v>
+        <v>29.36248401629709</v>
       </c>
       <c r="F5">
-        <v>16.2031869072372</v>
+        <v>18.39994300745641</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1561,19 +1538,19 @@
         <v>25</v>
       </c>
       <c r="B6">
-        <v>18.15449699644671</v>
+        <v>3.404173560934445</v>
       </c>
       <c r="C6">
-        <v>12.03451212769218</v>
+        <v>3.658446568725746</v>
       </c>
       <c r="D6">
-        <v>46.82970687871733</v>
+        <v>6.400633411059783</v>
       </c>
       <c r="E6">
-        <v>29.36248401629709</v>
+        <v>13.77726587702849</v>
       </c>
       <c r="F6">
-        <v>18.39994300745641</v>
+        <v>11.18513700531286</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1581,19 +1558,19 @@
         <v>26</v>
       </c>
       <c r="B7">
-        <v>3.404173560934445</v>
+        <v>1.998352710653228</v>
       </c>
       <c r="C7">
-        <v>3.658446568725746</v>
+        <v>1.538449817132225</v>
       </c>
       <c r="D7">
-        <v>6.400633411059783</v>
+        <v>4.249454880230769</v>
       </c>
       <c r="E7">
-        <v>13.77726587702849</v>
+        <v>16.10080664633304</v>
       </c>
       <c r="F7">
-        <v>11.18513700531286</v>
+        <v>4.389046963922966</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1601,38 +1578,18 @@
         <v>27</v>
       </c>
       <c r="B8">
-        <v>1.998352710653228</v>
+        <v>45.1486014057981</v>
       </c>
       <c r="C8">
-        <v>1.538449817132225</v>
+        <v>59.2369489711885</v>
       </c>
       <c r="D8">
-        <v>4.249454880230769</v>
+        <v>8.339349331546222</v>
       </c>
       <c r="E8">
-        <v>16.10080664633304</v>
+        <v>8.80311570533306</v>
       </c>
       <c r="F8">
-        <v>4.389046963922966</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9">
-        <v>45.1486014057981</v>
-      </c>
-      <c r="C9">
-        <v>59.2369489711885</v>
-      </c>
-      <c r="D9">
-        <v>8.339349331546222</v>
-      </c>
-      <c r="E9">
-        <v>8.803115705333058</v>
-      </c>
-      <c r="F9">
         <v>46.10129550091488</v>
       </c>
     </row>

</xml_diff>